<commit_message>
Add backfill tool, market type tracking, update JSON/XLSX data and readme
</commit_message>
<xml_diff>
--- a/monitor_xlsx/20260123.xlsx
+++ b/monitor_xlsx/20260123.xlsx
@@ -544,10 +544,6 @@
           <t>-0.21%</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -570,10 +566,6 @@
           <t>+1.37%</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -596,10 +588,6 @@
           <t>-0.19%</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr"/>
-      <c r="H6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -622,10 +610,6 @@
           <t>-1.21%</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr"/>
-      <c r="F7" t="inlineStr"/>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -648,10 +632,6 @@
           <t>+2.88%</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr"/>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -669,7 +649,6 @@
           <t>232.09億</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
           <t>-67.72億</t>
@@ -707,7 +686,6 @@
           <t>-8.38億</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
           <t>-84.37億</t>
@@ -718,8 +696,6 @@
           <t>-421.86億</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr"/>
-      <c r="H10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -737,15 +713,11 @@
           <t>149.5%</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
           <t>155.95%</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr"/>
-      <c r="G11" t="inlineStr"/>
-      <c r="H11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -763,11 +735,6 @@
           <t>270.58億</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr"/>
-      <c r="E12" t="inlineStr"/>
-      <c r="F12" t="inlineStr"/>
-      <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -785,15 +752,11 @@
           <t>8819口</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
           <t>13881口</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr"/>
-      <c r="G13" t="inlineStr"/>
-      <c r="H13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -811,7 +774,6 @@
           <t>-49.36億</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
           <t>-30.28億</t>
@@ -916,10 +878,6 @@
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" t="inlineStr"/>
-      <c r="B8" t="inlineStr"/>
-    </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
@@ -1041,7 +999,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V19"/>
+  <dimension ref="A1:V21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1058,7 +1016,7 @@
     <col width="12" customWidth="1" min="12" max="12"/>
     <col width="12" customWidth="1" min="13" max="13"/>
     <col width="12" customWidth="1" min="14" max="14"/>
-    <col width="14" customWidth="1" min="15" max="15"/>
+    <col width="12" customWidth="1" min="15" max="15"/>
     <col width="12" customWidth="1" min="16" max="16"/>
     <col width="14" customWidth="1" min="17" max="17"/>
     <col width="14" customWidth="1" min="18" max="18"/>
@@ -1075,6 +1033,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
@@ -2094,6 +2053,112 @@
       <c r="V19" t="inlineStr">
         <is>
           <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>6669</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>緯穎</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>3695</v>
+      </c>
+      <c r="D20" t="n">
+        <v>-1.86</v>
+      </c>
+      <c r="E20" t="n">
+        <v>1646</v>
+      </c>
+      <c r="F20" s="6" t="n">
+        <v>-145</v>
+      </c>
+      <c r="G20" t="n">
+        <v>-483</v>
+      </c>
+      <c r="H20" t="n">
+        <v>-212</v>
+      </c>
+      <c r="I20" t="n">
+        <v>-106</v>
+      </c>
+      <c r="J20" t="n">
+        <v>47</v>
+      </c>
+      <c r="K20" t="n">
+        <v>2377</v>
+      </c>
+      <c r="L20" t="n">
+        <v>9785</v>
+      </c>
+      <c r="M20" t="n">
+        <v>-46410</v>
+      </c>
+      <c r="N20" t="n">
+        <v>-18.67</v>
+      </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>主力積極賣出</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>3138</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>耀登</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>173</v>
+      </c>
+      <c r="D21" s="7" t="n">
+        <v>-1.14</v>
+      </c>
+      <c r="E21" t="n">
+        <v>1759</v>
+      </c>
+      <c r="F21" s="7" t="n">
+        <v>114</v>
+      </c>
+      <c r="G21" t="n">
+        <v>289</v>
+      </c>
+      <c r="H21" t="n">
+        <v>0</v>
+      </c>
+      <c r="I21" t="n">
+        <v>0</v>
+      </c>
+      <c r="J21" t="n">
+        <v>1</v>
+      </c>
+      <c r="K21" t="n">
+        <v>3626</v>
+      </c>
+      <c r="L21" t="n">
+        <v>17714</v>
+      </c>
+      <c r="M21" t="n">
+        <v>-11346</v>
+      </c>
+      <c r="N21" t="n">
+        <v>4.13</v>
+      </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>偏多</t>
         </is>
       </c>
     </row>

</xml_diff>